<commit_message>
chore: deploy updated fp test set 0 workbook
</commit_message>
<xml_diff>
--- a/fixtures/fp-tests/0.xlsx
+++ b/fixtures/fp-tests/0.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10621"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334C0193-F902-C44E-9EDE-934C615BD911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11D690A-734A-F64A-88CF-DAA8079BB0BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="26360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="217">
   <si>
     <t>Floor Name</t>
   </si>
@@ -439,15 +439,63 @@
     <t>Second Floor</t>
   </si>
   <si>
+    <t>16.B.048.TH</t>
+  </si>
+  <si>
+    <t>16.B.050.TH</t>
+  </si>
+  <si>
+    <t>16.B.051.TH</t>
+  </si>
+  <si>
+    <t>16.B.049.TH</t>
+  </si>
+  <si>
+    <t>16.B.052.TH</t>
+  </si>
+  <si>
+    <t>16.B.044.TH</t>
+  </si>
+  <si>
+    <t>16.B.046.TH</t>
+  </si>
+  <si>
     <t>16.B.058.TH</t>
   </si>
   <si>
+    <t>16.B.045.TH</t>
+  </si>
+  <si>
+    <t>16.B.055.TH</t>
+  </si>
+  <si>
     <t>16.B.057.TH</t>
   </si>
   <si>
+    <t>16.B.028.TH</t>
+  </si>
+  <si>
+    <t>16.B.056.TH</t>
+  </si>
+  <si>
+    <t>16.B.030.TH</t>
+  </si>
+  <si>
+    <t>16.B.026.TH</t>
+  </si>
+  <si>
+    <t>16.B.025.TH</t>
+  </si>
+  <si>
+    <t>16.B.027.TH</t>
+  </si>
+  <si>
     <t>16.B.064.TH</t>
   </si>
   <si>
+    <t>16.B.024.TH</t>
+  </si>
+  <si>
     <t>16.B.065.TH</t>
   </si>
   <si>
@@ -466,18 +514,72 @@
     <t>16.B.070.TH</t>
   </si>
   <si>
+    <t>16.B.036.TH</t>
+  </si>
+  <si>
+    <t>16.B.035.TH</t>
+  </si>
+  <si>
+    <t>16.B.037.TH</t>
+  </si>
+  <si>
+    <t>16.B.034.TH</t>
+  </si>
+  <si>
+    <t>16.B.043.TH</t>
+  </si>
+  <si>
+    <t>16.B.032.TH</t>
+  </si>
+  <si>
+    <t>16.B.038.TH</t>
+  </si>
+  <si>
+    <t>16.B.042.TH</t>
+  </si>
+  <si>
+    <t>16.B.039.TH</t>
+  </si>
+  <si>
+    <t>16.B.040.TH</t>
+  </si>
+  <si>
     <t>16.B.087.TH</t>
   </si>
   <si>
+    <t>16.B.053.TH</t>
+  </si>
+  <si>
     <t>16.B.088.TH</t>
   </si>
   <si>
+    <t>16.B.029.TH</t>
+  </si>
+  <si>
+    <t>16.B.031.TH</t>
+  </si>
+  <si>
+    <t>16.B.054.TH</t>
+  </si>
+  <si>
+    <t>16.B.022.TH</t>
+  </si>
+  <si>
+    <t>16.B.041.TH</t>
+  </si>
+  <si>
+    <t>16.B.047.TH</t>
+  </si>
+  <si>
     <t>16.B.067.TH</t>
   </si>
   <si>
     <t>16.B.089.TH</t>
   </si>
   <si>
+    <t>16.B.033.TH</t>
+  </si>
+  <si>
     <t>16.B.059.TH</t>
   </si>
   <si>
@@ -485,6 +587,57 @@
   </si>
   <si>
     <t>16.B.085.TH</t>
+  </si>
+  <si>
+    <t>16.B.015.TH</t>
+  </si>
+  <si>
+    <t>16.B.016.TH</t>
+  </si>
+  <si>
+    <t>16.B.001.TH</t>
+  </si>
+  <si>
+    <t>16.B.002.TH</t>
+  </si>
+  <si>
+    <t>16.B.003.TH</t>
+  </si>
+  <si>
+    <t>16.B.004.TH</t>
+  </si>
+  <si>
+    <t>16.B.005.TH</t>
+  </si>
+  <si>
+    <t>16.B.006.TH</t>
+  </si>
+  <si>
+    <t>16.B.007.TH</t>
+  </si>
+  <si>
+    <t>16.B.008.TH</t>
+  </si>
+  <si>
+    <t>16.B.009.TH</t>
+  </si>
+  <si>
+    <t>16.B.017.TH</t>
+  </si>
+  <si>
+    <t>16.B.018.TH</t>
+  </si>
+  <si>
+    <t>16.B.019.TH</t>
+  </si>
+  <si>
+    <t>16.B.020.TH</t>
+  </si>
+  <si>
+    <t>16.B.021.TH</t>
+  </si>
+  <si>
+    <t>16.B.023.TH</t>
   </si>
   <si>
     <t>16.B.060.TH</t>
@@ -914,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -946,7 +1099,7 @@
         <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>187</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -960,7 +1113,7 @@
         <v>133</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -974,7 +1127,7 @@
         <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>189</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -988,7 +1141,7 @@
         <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1002,7 +1155,7 @@
         <v>133</v>
       </c>
       <c r="B6" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1016,7 +1169,7 @@
         <v>133</v>
       </c>
       <c r="B7" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1030,7 +1183,7 @@
         <v>133</v>
       </c>
       <c r="B8" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1044,7 +1197,7 @@
         <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>194</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1058,7 +1211,7 @@
         <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>195</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1072,7 +1225,7 @@
         <v>133</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1086,7 +1239,7 @@
         <v>133</v>
       </c>
       <c r="B12" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1100,7 +1253,7 @@
         <v>133</v>
       </c>
       <c r="B13" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1114,7 +1267,7 @@
         <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>143</v>
+        <v>197</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1128,7 +1281,7 @@
         <v>133</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>198</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1142,7 +1295,7 @@
         <v>133</v>
       </c>
       <c r="B16" t="s">
-        <v>141</v>
+        <v>199</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1156,7 +1309,7 @@
         <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1170,7 +1323,7 @@
         <v>133</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1184,7 +1337,7 @@
         <v>133</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>201</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1198,7 +1351,7 @@
         <v>133</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1212,7 +1365,7 @@
         <v>133</v>
       </c>
       <c r="B21" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1226,7 +1379,7 @@
         <v>133</v>
       </c>
       <c r="B22" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1240,7 +1393,7 @@
         <v>133</v>
       </c>
       <c r="B23" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1254,7 +1407,7 @@
         <v>133</v>
       </c>
       <c r="B24" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1268,7 +1421,7 @@
         <v>133</v>
       </c>
       <c r="B25" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1282,7 +1435,7 @@
         <v>133</v>
       </c>
       <c r="B26" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1296,7 +1449,7 @@
         <v>133</v>
       </c>
       <c r="B27" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1310,7 +1463,7 @@
         <v>133</v>
       </c>
       <c r="B28" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -1324,7 +1477,7 @@
         <v>133</v>
       </c>
       <c r="B29" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1352,7 +1505,7 @@
         <v>133</v>
       </c>
       <c r="B31" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1366,12 +1519,726 @@
         <v>133</v>
       </c>
       <c r="B32" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" t="s">
+        <v>162</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" t="s">
+        <v>166</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" t="s">
+        <v>168</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>133</v>
+      </c>
+      <c r="B36" t="s">
+        <v>169</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" t="s">
+        <v>177</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" t="s">
+        <v>167</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>133</v>
+      </c>
+      <c r="B39" t="s">
+        <v>164</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" t="s">
+        <v>140</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" t="s">
+        <v>143</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" t="s">
+        <v>141</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>133</v>
+      </c>
+      <c r="B43" t="s">
+        <v>178</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>133</v>
+      </c>
+      <c r="B44" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>133</v>
+      </c>
+      <c r="B46" t="s">
+        <v>136</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>133</v>
+      </c>
+      <c r="B47" t="s">
+        <v>137</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>133</v>
+      </c>
+      <c r="B48" t="s">
+        <v>139</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" t="s">
+        <v>171</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" t="s">
+        <v>175</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>133</v>
+      </c>
+      <c r="B51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" t="s">
+        <v>147</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>133</v>
+      </c>
+      <c r="B53" t="s">
+        <v>145</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>133</v>
+      </c>
+      <c r="B54" t="s">
+        <v>142</v>
+      </c>
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>133</v>
+      </c>
+      <c r="B55" t="s">
+        <v>182</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>133</v>
+      </c>
+      <c r="B56" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56">
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" t="s">
+        <v>203</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>133</v>
+      </c>
+      <c r="B58" t="s">
+        <v>204</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>133</v>
+      </c>
+      <c r="B59" t="s">
+        <v>205</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>133</v>
+      </c>
+      <c r="B60" t="s">
+        <v>152</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>133</v>
+      </c>
+      <c r="B61" t="s">
+        <v>154</v>
+      </c>
+      <c r="C61">
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>133</v>
+      </c>
+      <c r="B62" t="s">
+        <v>155</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>133</v>
+      </c>
+      <c r="B63" t="s">
+        <v>179</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>133</v>
+      </c>
+      <c r="B64" t="s">
+        <v>206</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>133</v>
+      </c>
+      <c r="B65" t="s">
+        <v>159</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>133</v>
+      </c>
+      <c r="B66" t="s">
+        <v>158</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" t="s">
+        <v>157</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>133</v>
+      </c>
+      <c r="B68" t="s">
+        <v>156</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>133</v>
+      </c>
+      <c r="B69" t="s">
+        <v>207</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>133</v>
+      </c>
+      <c r="B70" t="s">
+        <v>184</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>133</v>
+      </c>
+      <c r="B71" t="s">
+        <v>208</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>133</v>
+      </c>
+      <c r="B72" t="s">
+        <v>170</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>133</v>
+      </c>
+      <c r="B73" t="s">
+        <v>172</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>133</v>
+      </c>
+      <c r="B74" t="s">
+        <v>180</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>133</v>
+      </c>
+      <c r="B75" t="s">
+        <v>183</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>133</v>
+      </c>
+      <c r="B76" t="s">
+        <v>209</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>133</v>
+      </c>
+      <c r="B77" t="s">
+        <v>210</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>133</v>
+      </c>
+      <c r="B78" t="s">
+        <v>211</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>133</v>
+      </c>
+      <c r="B79" t="s">
+        <v>212</v>
+      </c>
+      <c r="C79">
+        <v>0</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>133</v>
+      </c>
+      <c r="B80" t="s">
+        <v>213</v>
+      </c>
+      <c r="C80">
+        <v>0</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>133</v>
+      </c>
+      <c r="B81" t="s">
+        <v>214</v>
+      </c>
+      <c r="C81">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>133</v>
+      </c>
+      <c r="B82" t="s">
+        <v>215</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>133</v>
+      </c>
+      <c r="B83" t="s">
+        <v>216</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+      <c r="D83">
         <v>0</v>
       </c>
     </row>

</xml_diff>